<commit_message>
Correct H2KG parameter-property semantics
</commit_message>
<xml_diff>
--- a/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
+++ b/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>107 (4.53%)</t>
+          <t>108 (4.58%)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>638 (27.03%)</t>
+          <t>637 (26.99%)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1439 (60.98%)</t>
+          <t>1439 (60.97%)</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>110 (4.66%)</t>
+          <t>111 (4.70%)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>550 (23.30%)</t>
+          <t>549 (23.26%)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>18 (0.76%)</t>
+          <t>19 (0.81%)</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>79 (3.35%)</t>
+          <t>78 (3.30%)</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="J132" s="4" t="inlineStr">
         <is>
-          <t>8 (0.34%)</t>
+          <t>9 (0.38%)</t>
         </is>
       </c>
       <c r="K132" s="4" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="L132" s="4" t="inlineStr">
         <is>
-          <t>4 (0.17%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="M132" s="4" t="inlineStr">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="J140" s="4" t="inlineStr">
         <is>
-          <t>29 (1.23%)</t>
+          <t>30 (1.27%)</t>
         </is>
       </c>
       <c r="K140" s="4" t="inlineStr">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="L140" s="4" t="inlineStr">
         <is>
-          <t>101 (4.28%)</t>
+          <t>100 (4.24%)</t>
         </is>
       </c>
       <c r="M140" s="4" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="J150" s="4" t="inlineStr">
         <is>
-          <t>18 (0.76%)</t>
+          <t>19 (0.81%)</t>
         </is>
       </c>
       <c r="K150" s="4" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="L150" s="4" t="inlineStr">
         <is>
-          <t>79 (3.35%)</t>
+          <t>78 (3.30%)</t>
         </is>
       </c>
       <c r="M150" s="4" t="inlineStr">
@@ -11593,7 +11593,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1171</v>
+        <v>1176</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -11605,25 +11605,25 @@
         <v>18</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>1.5371</v>
+        <v>1.5306</v>
       </c>
       <c r="H3" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I3" s="8" t="n">
-        <v>5.2092</v>
+        <v>5.2721</v>
       </c>
       <c r="J3" t="n">
         <v>21</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>1.7933</v>
+        <v>1.7857</v>
       </c>
       <c r="L3" t="n">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="M3" s="8" t="n">
-        <v>28.0102</v>
+        <v>27.9762</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -11632,10 +11632,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="Q3" s="8" t="n">
-        <v>63.45</v>
+        <v>63.4354</v>
       </c>
     </row>
     <row r="4">
@@ -11650,7 +11650,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -11662,25 +11662,25 @@
         <v>1</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.8621</v>
+        <v>0.9091</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>2.5862</v>
+        <v>2.7273</v>
       </c>
       <c r="J4" t="n">
         <v>6</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>5.1724</v>
+        <v>5.4545</v>
       </c>
       <c r="L4" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>26.7241</v>
+        <v>26.3636</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -11689,10 +11689,10 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="Q4" s="8" t="n">
-        <v>64.65519999999999</v>
+        <v>64.5455</v>
       </c>
     </row>
     <row r="5">
@@ -11707,7 +11707,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -11719,25 +11719,25 @@
         <v>39</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>5.5398</v>
+        <v>5.5319</v>
       </c>
       <c r="H5" t="n">
         <v>25</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>3.5511</v>
+        <v>3.5461</v>
       </c>
       <c r="J5" t="n">
         <v>44</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>6.25</v>
+        <v>6.2411</v>
       </c>
       <c r="L5" t="n">
         <v>186</v>
       </c>
       <c r="M5" s="8" t="n">
-        <v>26.4205</v>
+        <v>26.383</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -11746,10 +11746,10 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="Q5" s="8" t="n">
-        <v>58.2386</v>
+        <v>58.2979</v>
       </c>
     </row>
     <row r="6">
@@ -11878,7 +11878,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1171</v>
+        <v>1176</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -11896,19 +11896,19 @@
         <v>11</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>0.9394</v>
+        <v>0.9354</v>
       </c>
       <c r="J8" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>0.3416</v>
+        <v>0.3401</v>
       </c>
       <c r="L8" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>10.9308</v>
+        <v>10.9694</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -11917,10 +11917,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>87.7882</v>
+        <v>87.7551</v>
       </c>
     </row>
     <row r="9">
@@ -11935,7 +11935,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -11947,7 +11947,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.8621</v>
+        <v>0.9091</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -11962,10 +11962,10 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>12.931</v>
+        <v>12.7273</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
@@ -11974,10 +11974,10 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>86.2069</v>
+        <v>86.36360000000001</v>
       </c>
     </row>
     <row r="10">
@@ -11992,7 +11992,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -12004,25 +12004,25 @@
         <v>5</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.7102000000000001</v>
+        <v>0.7092000000000001</v>
       </c>
       <c r="H10" t="n">
         <v>4</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>0.5682</v>
+        <v>0.5674</v>
       </c>
       <c r="J10" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>0.7102000000000001</v>
+        <v>0.7092000000000001</v>
       </c>
       <c r="L10" t="n">
         <v>45</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>6.392</v>
+        <v>6.383</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -12031,10 +12031,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>91.6193</v>
+        <v>91.63120000000001</v>
       </c>
     </row>
     <row r="11">
@@ -12163,7 +12163,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1171</v>
+        <v>1176</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -12175,25 +12175,25 @@
         <v>17</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>1.4518</v>
+        <v>1.4456</v>
       </c>
       <c r="H13" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>6.234</v>
+        <v>6.2925</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>1.7079</v>
+        <v>1.7007</v>
       </c>
       <c r="L13" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>25.2775</v>
+        <v>25.2551</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -12202,10 +12202,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>65.3288</v>
+        <v>65.3061</v>
       </c>
     </row>
     <row r="14">
@@ -12220,7 +12220,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -12232,25 +12232,25 @@
         <v>3</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>2.5862</v>
+        <v>2.7273</v>
       </c>
       <c r="H14" t="n">
         <v>5</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>4.3103</v>
+        <v>4.5455</v>
       </c>
       <c r="J14" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>2.5862</v>
+        <v>2.7273</v>
       </c>
       <c r="L14" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="M14" s="8" t="n">
-        <v>24.1379</v>
+        <v>23.6364</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -12259,10 +12259,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>66.3793</v>
+        <v>66.36360000000001</v>
       </c>
     </row>
     <row r="15">
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -12289,25 +12289,25 @@
         <v>16</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>2.2727</v>
+        <v>2.2695</v>
       </c>
       <c r="H15" t="n">
         <v>13</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>1.8466</v>
+        <v>1.844</v>
       </c>
       <c r="J15" t="n">
         <v>12</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>1.7045</v>
+        <v>1.7021</v>
       </c>
       <c r="L15" t="n">
         <v>123</v>
       </c>
       <c r="M15" s="8" t="n">
-        <v>17.4716</v>
+        <v>17.4468</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -12316,10 +12316,10 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="Q15" s="8" t="n">
-        <v>76.7045</v>
+        <v>76.7376</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Sanitize synthetic TEM evidence and benchmark metadata
</commit_message>
<xml_diff>
--- a/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
+++ b/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Collection summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ontology benchmark" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="H2KG branch summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ontology benchmark" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="H2KG branch summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Collection summary'!$A$1:$J$4</definedName>

</xml_diff>

<commit_message>
Correct H2KG evaluation and DECODE semantics
</commit_message>
<xml_diff>
--- a/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
+++ b/ontology_release/output/benchmarks/tib_collections/h2kg_tib_manuscript_tables.xlsx
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="4">
@@ -691,7 +691,7 @@
         <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -700,22 +700,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>88 (3.96%)</t>
+          <t>88 (3.95%)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>103 (4.64%)</t>
+          <t>103 (4.63%)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>85 (3.83%)</t>
+          <t>85 (3.82%)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>601 (27.06%)</t>
+          <t>601 (27.00%)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1344 (60.51%)</t>
+          <t>1349 (60.60%)</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
         <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>196 (8.82%)</t>
+          <t>196 (8.81%)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1989 (89.55%)</t>
+          <t>1994 (89.58%)</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
         <v>113</v>
       </c>
       <c r="D4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -807,17 +807,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>107 (4.82%)</t>
+          <t>107 (4.81%)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>45 (2.03%)</t>
+          <t>45 (2.02%)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>523 (23.55%)</t>
+          <t>523 (23.50%)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1496 (67.36%)</t>
+          <t>1501 (67.43%)</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>189 (8.51%)</t>
+          <t>189 (8.49%)</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>1970 (88.70%)</t>
+          <t>1975 (88.72%)</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
         </is>
       </c>
       <c r="I3" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>19 (0.86%)</t>
+          <t>19 (0.85%)</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>196 (8.82%)</t>
+          <t>196 (8.81%)</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="P4" s="4" t="inlineStr">
         <is>
-          <t>1991 (89.64%)</t>
+          <t>1996 (89.67%)</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="I5" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>2157 (97.12%)</t>
+          <t>2162 (97.12%)</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
@@ -1287,22 +1287,22 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>25 (1.13%)</t>
+          <t>25 (1.12%)</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>27 (1.22%)</t>
+          <t>27 (1.21%)</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>198 (8.91%)</t>
+          <t>198 (8.89%)</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>1964 (88.43%)</t>
+          <t>1969 (88.45%)</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>2203 (99.19%)</t>
+          <t>2208 (99.19%)</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>17 (0.77%)</t>
+          <t>17 (0.76%)</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>255 (11.48%)</t>
+          <t>255 (11.46%)</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>1889 (85.05%)</t>
+          <t>1894 (85.09%)</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1663,12 +1663,12 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>95 (4.28%)</t>
+          <t>95 (4.27%)</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>2111 (95.05%)</t>
+          <t>2116 (95.06%)</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>9 (0.41%)</t>
+          <t>9 (0.40%)</t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>11 (0.50%)</t>
+          <t>11 (0.49%)</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>189 (8.51%)</t>
+          <t>189 (8.49%)</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>2011 (90.54%)</t>
+          <t>2016 (90.57%)</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
         </is>
       </c>
       <c r="I13" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
@@ -1877,12 +1877,12 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>47 (2.12%)</t>
+          <t>47 (2.11%)</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>2173 (97.84%)</t>
+          <t>2178 (97.84%)</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="I15" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1951,12 +1951,12 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>19 (0.86%)</t>
+          <t>19 (0.85%)</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>183 (8.24%)</t>
+          <t>183 (8.22%)</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
-          <t>2005 (90.27%)</t>
+          <t>2010 (90.30%)</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="I17" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>93 (4.19%)</t>
+          <t>93 (4.18%)</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
@@ -2188,7 +2188,7 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>2108 (94.91%)</t>
+          <t>2113 (94.92%)</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>49 (2.21%)</t>
+          <t>49 (2.20%)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>2167 (97.57%)</t>
+          <t>2172 (97.57%)</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>2198 (98.96%)</t>
+          <t>2203 (98.97%)</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="I21" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>2211 (99.55%)</t>
+          <t>2216 (99.55%)</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="I22" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -2461,12 +2461,12 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>13 (0.59%)</t>
+          <t>13 (0.58%)</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>117 (5.27%)</t>
+          <t>117 (5.26%)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>2073 (93.34%)</t>
+          <t>2078 (93.35%)</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="I23" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>61 (2.75%)</t>
+          <t>61 (2.74%)</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>2146 (96.62%)</t>
+          <t>2151 (96.63%)</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="I24" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>72 (3.24%)</t>
+          <t>72 (3.23%)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>2128 (95.81%)</t>
+          <t>2133 (95.82%)</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
         </is>
       </c>
       <c r="I25" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>17 (0.77%)</t>
+          <t>17 (0.76%)</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>178 (8.01%)</t>
+          <t>178 (8.00%)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>1980 (89.15%)</t>
+          <t>1985 (89.17%)</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         </is>
       </c>
       <c r="I26" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>63 (2.84%)</t>
+          <t>63 (2.83%)</t>
         </is>
       </c>
       <c r="O26" s="7" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>2156 (97.07%)</t>
+          <t>2161 (97.08%)</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
         </is>
       </c>
       <c r="I27" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>2207 (99.37%)</t>
+          <t>2212 (99.37%)</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="I28" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="I29" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
         </is>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O30" s="7" t="inlineStr">
@@ -3060,7 +3060,7 @@
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="I31" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
@@ -3134,7 +3134,7 @@
       </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
         </is>
       </c>
       <c r="I32" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
         </is>
       </c>
       <c r="I33" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
       <c r="I34" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
         </is>
       </c>
       <c r="I35" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="I36" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="O36" s="7" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="I37" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
         </is>
       </c>
       <c r="I38" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3672,7 @@
         </is>
       </c>
       <c r="I39" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="I40" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="P40" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="I41" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
         </is>
       </c>
       <c r="I42" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
       <c r="I43" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="I44" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
@@ -4043,12 +4043,12 @@
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>102 (4.59%)</t>
+          <t>102 (4.58%)</t>
         </is>
       </c>
       <c r="O44" s="7" t="inlineStr">
@@ -4068,7 +4068,7 @@
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>2089 (94.06%)</t>
+          <t>2094 (94.07%)</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="I45" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
         </is>
       </c>
       <c r="I46" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
@@ -4187,7 +4187,7 @@
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="I47" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O47" s="7" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="I48" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
@@ -4340,7 +4340,7 @@
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="N48" s="7" t="inlineStr">
         <is>
-          <t>13 (0.59%)</t>
+          <t>13 (0.58%)</t>
         </is>
       </c>
       <c r="O48" s="7" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="P48" s="7" t="inlineStr">
         <is>
-          <t>2205 (99.28%)</t>
+          <t>2210 (99.28%)</t>
         </is>
       </c>
     </row>
@@ -4396,7 +4396,7 @@
         </is>
       </c>
       <c r="I49" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
         </is>
       </c>
       <c r="I50" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="I51" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>113 (5.09%)</t>
+          <t>113 (5.08%)</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>2108 (94.91%)</t>
+          <t>2113 (94.92%)</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
         </is>
       </c>
       <c r="I52" s="7" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
         </is>
       </c>
       <c r="I53" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
@@ -4711,12 +4711,12 @@
       </c>
       <c r="M53" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N53" s="4" t="inlineStr">
         <is>
-          <t>13 (0.59%)</t>
+          <t>13 (0.58%)</t>
         </is>
       </c>
       <c r="O53" s="4" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>2207 (99.37%)</t>
+          <t>2212 (99.37%)</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
         </is>
       </c>
       <c r="I54" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="P54" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
         </is>
       </c>
       <c r="I55" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="N55" s="4" t="inlineStr">
         <is>
-          <t>189 (8.51%)</t>
+          <t>189 (8.49%)</t>
         </is>
       </c>
       <c r="O55" s="4" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>1970 (88.70%)</t>
+          <t>1975 (88.72%)</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
         </is>
       </c>
       <c r="I56" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O56" s="4" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="P56" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="I57" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="N57" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O57" s="4" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="P57" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="I58" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="P58" s="4" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
         </is>
       </c>
       <c r="I59" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="P59" s="4" t="inlineStr">
         <is>
-          <t>2195 (98.83%)</t>
+          <t>2200 (98.83%)</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="N61" s="4" t="inlineStr">
         <is>
-          <t>63 (2.84%)</t>
+          <t>63 (2.83%)</t>
         </is>
       </c>
       <c r="O61" s="4" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="P61" s="4" t="inlineStr">
         <is>
-          <t>2156 (97.07%)</t>
+          <t>2161 (97.08%)</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
@@ -5350,7 +5350,7 @@
       </c>
       <c r="P62" s="4" t="inlineStr">
         <is>
-          <t>2211 (99.55%)</t>
+          <t>2216 (99.55%)</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="P63" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
         </is>
       </c>
       <c r="I64" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="L64" s="4" t="inlineStr">
@@ -5483,12 +5483,12 @@
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="N64" s="4" t="inlineStr">
         <is>
-          <t>55 (2.48%)</t>
+          <t>55 (2.47%)</t>
         </is>
       </c>
       <c r="O64" s="4" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="P64" s="4" t="inlineStr">
         <is>
-          <t>2148 (96.71%)</t>
+          <t>2153 (96.72%)</t>
         </is>
       </c>
     </row>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="I65" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="N65" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="O65" s="4" t="inlineStr">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="P65" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
         </is>
       </c>
       <c r="I66" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
@@ -5627,7 +5627,7 @@
       </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N66" s="4" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="P66" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
         </is>
       </c>
       <c r="I67" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="P67" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5756,7 @@
         </is>
       </c>
       <c r="I68" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
@@ -5780,7 +5780,7 @@
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>39 (1.76%)</t>
+          <t>39 (1.75%)</t>
         </is>
       </c>
       <c r="O68" s="4" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="P68" s="4" t="inlineStr">
         <is>
-          <t>2180 (98.15%)</t>
+          <t>2185 (98.16%)</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
         </is>
       </c>
       <c r="I69" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
         </is>
       </c>
       <c r="I70" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
@@ -5930,7 +5930,7 @@
       </c>
       <c r="P70" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -5970,7 +5970,7 @@
         </is>
       </c>
       <c r="I71" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="N71" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="O71" s="4" t="inlineStr">
@@ -6004,7 +6004,7 @@
       </c>
       <c r="P71" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6044,7 @@
         </is>
       </c>
       <c r="I72" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
@@ -6068,7 +6068,7 @@
       </c>
       <c r="N72" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="O72" s="4" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="P72" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="I73" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="P73" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -6188,7 +6188,7 @@
         </is>
       </c>
       <c r="I74" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="P74" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="P75" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
@@ -6341,22 +6341,22 @@
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M76" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="N76" s="4" t="inlineStr">
         <is>
-          <t>73 (3.29%)</t>
+          <t>73 (3.28%)</t>
         </is>
       </c>
       <c r="O76" s="4" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="P76" s="4" t="inlineStr">
         <is>
-          <t>2143 (96.49%)</t>
+          <t>2148 (96.50%)</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="I77" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
       </c>
       <c r="N77" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O77" s="4" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="P77" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
         </is>
       </c>
       <c r="I78" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
@@ -6499,12 +6499,12 @@
       </c>
       <c r="M78" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="N78" s="4" t="inlineStr">
         <is>
-          <t>95 (4.28%)</t>
+          <t>95 (4.27%)</t>
         </is>
       </c>
       <c r="O78" s="4" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="P78" s="4" t="inlineStr">
         <is>
-          <t>2111 (95.05%)</t>
+          <t>2116 (95.06%)</t>
         </is>
       </c>
     </row>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="I79" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
@@ -6584,7 +6584,7 @@
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="P80" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -6694,7 +6694,7 @@
         </is>
       </c>
       <c r="I81" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
@@ -6713,12 +6713,12 @@
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="N81" s="4" t="inlineStr">
         <is>
-          <t>29 (1.31%)</t>
+          <t>29 (1.30%)</t>
         </is>
       </c>
       <c r="O81" s="4" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="P81" s="4" t="inlineStr">
         <is>
-          <t>2189 (98.56%)</t>
+          <t>2194 (98.56%)</t>
         </is>
       </c>
     </row>
@@ -6764,7 +6764,7 @@
         </is>
       </c>
       <c r="I82" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="N82" s="4" t="inlineStr">
         <is>
-          <t>225 (10.13%)</t>
+          <t>225 (10.11%)</t>
         </is>
       </c>
       <c r="O82" s="4" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="P82" s="4" t="inlineStr">
         <is>
-          <t>1996 (89.87%)</t>
+          <t>2001 (89.89%)</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
         </is>
       </c>
       <c r="I83" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
@@ -6868,7 +6868,7 @@
       </c>
       <c r="P83" s="4" t="inlineStr">
         <is>
-          <t>2181 (98.20%)</t>
+          <t>2186 (98.20%)</t>
         </is>
       </c>
     </row>
@@ -6904,7 +6904,7 @@
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="P84" s="4" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
         </is>
       </c>
       <c r="I85" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
@@ -6988,7 +6988,7 @@
       </c>
       <c r="L85" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M85" s="4" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="P85" s="4" t="inlineStr">
         <is>
-          <t>2202 (99.14%)</t>
+          <t>2207 (99.15%)</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
         </is>
       </c>
       <c r="I86" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
       </c>
       <c r="L86" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="P86" s="4" t="inlineStr">
         <is>
-          <t>2210 (99.50%)</t>
+          <t>2215 (99.51%)</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7120,7 @@
         </is>
       </c>
       <c r="I87" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="P87" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7190,7 +7190,7 @@
         </is>
       </c>
       <c r="I88" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="N88" s="4" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="O88" s="4" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="P88" s="4" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7260,7 @@
         </is>
       </c>
       <c r="I89" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
@@ -7294,7 +7294,7 @@
       </c>
       <c r="P89" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7330,7 +7330,7 @@
         </is>
       </c>
       <c r="I90" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
@@ -7344,7 +7344,7 @@
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="M90" s="4" t="inlineStr">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="P90" s="4" t="inlineStr">
         <is>
-          <t>2210 (99.50%)</t>
+          <t>2215 (99.51%)</t>
         </is>
       </c>
     </row>
@@ -7400,7 +7400,7 @@
         </is>
       </c>
       <c r="I91" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="P91" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7470,7 +7470,7 @@
         </is>
       </c>
       <c r="I92" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="P92" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
         </is>
       </c>
       <c r="I93" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M93" s="4" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="N93" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="O93" s="4" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="P93" s="4" t="inlineStr">
         <is>
-          <t>2215 (99.73%)</t>
+          <t>2220 (99.73%)</t>
         </is>
       </c>
     </row>
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="I94" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="P94" s="4" t="inlineStr">
         <is>
-          <t>2205 (99.28%)</t>
+          <t>2210 (99.28%)</t>
         </is>
       </c>
     </row>
@@ -7688,7 +7688,7 @@
         </is>
       </c>
       <c r="I95" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
@@ -7697,7 +7697,7 @@
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L95" s="4" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="N95" s="4" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="O95" s="4" t="inlineStr">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="P95" s="4" t="inlineStr">
         <is>
-          <t>2203 (99.19%)</t>
+          <t>2208 (99.19%)</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="I96" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="P96" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7832,7 @@
         </is>
       </c>
       <c r="I97" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J97" s="4" t="inlineStr">
         <is>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="P97" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
         </is>
       </c>
       <c r="I98" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="P98" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
         </is>
       </c>
       <c r="I99" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="N99" s="4" t="inlineStr">
         <is>
-          <t>11 (0.50%)</t>
+          <t>11 (0.49%)</t>
         </is>
       </c>
       <c r="O99" s="4" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="P99" s="4" t="inlineStr">
         <is>
-          <t>2210 (99.50%)</t>
+          <t>2215 (99.51%)</t>
         </is>
       </c>
     </row>
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="I100" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J100" s="4" t="inlineStr">
         <is>
@@ -8074,7 +8074,7 @@
       </c>
       <c r="N100" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O100" s="4" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="P100" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
         </is>
       </c>
       <c r="I101" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J101" s="4" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
       </c>
       <c r="N101" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="O101" s="4" t="inlineStr">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="P101" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8194,7 @@
         </is>
       </c>
       <c r="I102" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J102" s="4" t="inlineStr">
         <is>
@@ -8213,7 +8213,7 @@
       </c>
       <c r="M102" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N102" s="4" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="P102" s="4" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="I103" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J103" s="4" t="inlineStr">
         <is>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="P103" s="4" t="inlineStr">
         <is>
-          <t>2191 (98.65%)</t>
+          <t>2196 (98.65%)</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
         </is>
       </c>
       <c r="I104" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J104" s="4" t="inlineStr">
         <is>
@@ -8376,7 +8376,7 @@
       </c>
       <c r="P104" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8416,7 @@
         </is>
       </c>
       <c r="I105" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J105" s="4" t="inlineStr">
         <is>
@@ -8450,7 +8450,7 @@
       </c>
       <c r="P105" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="I106" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J106" s="4" t="inlineStr">
         <is>
@@ -8514,7 +8514,7 @@
       </c>
       <c r="N106" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O106" s="4" t="inlineStr">
@@ -8524,7 +8524,7 @@
       </c>
       <c r="P106" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
         </is>
       </c>
       <c r="I107" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="N107" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="O107" s="4" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="P107" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -8638,7 +8638,7 @@
         </is>
       </c>
       <c r="I108" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
@@ -8672,7 +8672,7 @@
       </c>
       <c r="P108" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="I109" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
@@ -8721,7 +8721,7 @@
       </c>
       <c r="K109" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L109" s="4" t="inlineStr">
@@ -8731,12 +8731,12 @@
       </c>
       <c r="M109" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N109" s="4" t="inlineStr">
         <is>
-          <t>11 (0.50%)</t>
+          <t>11 (0.49%)</t>
         </is>
       </c>
       <c r="O109" s="4" t="inlineStr">
@@ -8746,7 +8746,7 @@
       </c>
       <c r="P109" s="4" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -8786,7 +8786,7 @@
         </is>
       </c>
       <c r="I110" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J110" s="4" t="inlineStr">
         <is>
@@ -8795,7 +8795,7 @@
       </c>
       <c r="K110" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="L110" s="4" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="P110" s="4" t="inlineStr">
         <is>
-          <t>2202 (99.14%)</t>
+          <t>2207 (99.15%)</t>
         </is>
       </c>
     </row>
@@ -8856,7 +8856,7 @@
         </is>
       </c>
       <c r="I111" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J111" s="4" t="inlineStr">
         <is>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="P111" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -8930,7 +8930,7 @@
         </is>
       </c>
       <c r="I112" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J112" s="4" t="inlineStr">
         <is>
@@ -8939,7 +8939,7 @@
       </c>
       <c r="K112" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L112" s="4" t="inlineStr">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="P112" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
         </is>
       </c>
       <c r="I113" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J113" s="4" t="inlineStr">
         <is>
@@ -9028,7 +9028,7 @@
       </c>
       <c r="N113" s="4" t="inlineStr">
         <is>
-          <t>93 (4.19%)</t>
+          <t>93 (4.18%)</t>
         </is>
       </c>
       <c r="O113" s="4" t="inlineStr">
@@ -9038,7 +9038,7 @@
       </c>
       <c r="P113" s="4" t="inlineStr">
         <is>
-          <t>2108 (94.91%)</t>
+          <t>2113 (94.92%)</t>
         </is>
       </c>
     </row>
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="I114" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J114" s="4" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
       </c>
       <c r="N114" s="4" t="inlineStr">
         <is>
-          <t>219 (9.86%)</t>
+          <t>219 (9.84%)</t>
         </is>
       </c>
       <c r="O114" s="4" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="P114" s="4" t="inlineStr">
         <is>
-          <t>2002 (90.14%)</t>
+          <t>2007 (90.16%)</t>
         </is>
       </c>
     </row>
@@ -9148,7 +9148,7 @@
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J115" s="4" t="inlineStr">
         <is>
@@ -9157,12 +9157,12 @@
       </c>
       <c r="K115" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="L115" s="4" t="inlineStr">
         <is>
-          <t>23 (1.04%)</t>
+          <t>23 (1.03%)</t>
         </is>
       </c>
       <c r="M115" s="4" t="inlineStr">
@@ -9172,7 +9172,7 @@
       </c>
       <c r="N115" s="4" t="inlineStr">
         <is>
-          <t>210 (9.46%)</t>
+          <t>210 (9.43%)</t>
         </is>
       </c>
       <c r="O115" s="4" t="inlineStr">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="P115" s="4" t="inlineStr">
         <is>
-          <t>1979 (89.10%)</t>
+          <t>1984 (89.13%)</t>
         </is>
       </c>
     </row>
@@ -9222,7 +9222,7 @@
         </is>
       </c>
       <c r="I116" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J116" s="4" t="inlineStr">
         <is>
@@ -9241,7 +9241,7 @@
       </c>
       <c r="M116" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N116" s="4" t="inlineStr">
@@ -9256,7 +9256,7 @@
       </c>
       <c r="P116" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -9292,7 +9292,7 @@
         </is>
       </c>
       <c r="I117" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J117" s="4" t="inlineStr">
         <is>
@@ -9326,7 +9326,7 @@
       </c>
       <c r="P117" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="I118" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J118" s="4" t="inlineStr">
         <is>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="P118" s="4" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -9432,7 +9432,7 @@
         </is>
       </c>
       <c r="I119" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J119" s="4" t="inlineStr">
         <is>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="N119" s="4" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="O119" s="4" t="inlineStr">
@@ -9466,7 +9466,7 @@
       </c>
       <c r="P119" s="4" t="inlineStr">
         <is>
-          <t>2206 (99.32%)</t>
+          <t>2211 (99.33%)</t>
         </is>
       </c>
     </row>
@@ -9506,7 +9506,7 @@
         </is>
       </c>
       <c r="I120" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J120" s="4" t="inlineStr">
         <is>
@@ -9540,7 +9540,7 @@
       </c>
       <c r="P120" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9576,7 @@
         </is>
       </c>
       <c r="I121" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J121" s="4" t="inlineStr">
         <is>
@@ -9610,7 +9610,7 @@
       </c>
       <c r="P121" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9646,7 @@
         </is>
       </c>
       <c r="I122" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J122" s="4" t="inlineStr">
         <is>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="P122" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9720,7 +9720,7 @@
         </is>
       </c>
       <c r="I123" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J123" s="4" t="inlineStr">
         <is>
@@ -9754,7 +9754,7 @@
       </c>
       <c r="P123" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9794,7 @@
         </is>
       </c>
       <c r="I124" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J124" s="4" t="inlineStr">
         <is>
@@ -9828,7 +9828,7 @@
       </c>
       <c r="P124" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9864,7 +9864,7 @@
         </is>
       </c>
       <c r="I125" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J125" s="4" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
       </c>
       <c r="P125" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -9934,7 +9934,7 @@
         </is>
       </c>
       <c r="I126" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J126" s="4" t="inlineStr">
         <is>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="N126" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O126" s="4" t="inlineStr">
@@ -9968,7 +9968,7 @@
       </c>
       <c r="P126" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -10008,7 +10008,7 @@
         </is>
       </c>
       <c r="I127" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J127" s="4" t="inlineStr">
         <is>
@@ -10017,12 +10017,12 @@
       </c>
       <c r="K127" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="L127" s="4" t="inlineStr">
         <is>
-          <t>15 (0.68%)</t>
+          <t>15 (0.67%)</t>
         </is>
       </c>
       <c r="M127" s="4" t="inlineStr">
@@ -10032,7 +10032,7 @@
       </c>
       <c r="N127" s="4" t="inlineStr">
         <is>
-          <t>102 (4.59%)</t>
+          <t>102 (4.58%)</t>
         </is>
       </c>
       <c r="O127" s="4" t="inlineStr">
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P127" s="4" t="inlineStr">
         <is>
-          <t>2089 (94.06%)</t>
+          <t>2094 (94.07%)</t>
         </is>
       </c>
     </row>
@@ -10082,7 +10082,7 @@
         </is>
       </c>
       <c r="I128" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J128" s="4" t="inlineStr">
         <is>
@@ -10091,7 +10091,7 @@
       </c>
       <c r="K128" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L128" s="4" t="inlineStr">
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P128" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -10156,7 +10156,7 @@
         </is>
       </c>
       <c r="I129" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J129" s="4" t="inlineStr">
         <is>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="P129" s="4" t="inlineStr">
         <is>
-          <t>2217 (99.82%)</t>
+          <t>2222 (99.82%)</t>
         </is>
       </c>
     </row>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="I130" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J130" s="4" t="inlineStr">
         <is>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="N130" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O130" s="4" t="inlineStr">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="P130" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -10304,7 +10304,7 @@
         </is>
       </c>
       <c r="I131" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J131" s="4" t="inlineStr">
         <is>
@@ -10338,7 +10338,7 @@
       </c>
       <c r="P131" s="4" t="inlineStr">
         <is>
-          <t>2217 (99.82%)</t>
+          <t>2222 (99.82%)</t>
         </is>
       </c>
     </row>
@@ -10378,7 +10378,7 @@
         </is>
       </c>
       <c r="I132" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J132" s="4" t="inlineStr">
         <is>
@@ -10392,7 +10392,7 @@
       </c>
       <c r="L132" s="4" t="inlineStr">
         <is>
-          <t>9 (0.41%)</t>
+          <t>9 (0.40%)</t>
         </is>
       </c>
       <c r="M132" s="4" t="inlineStr">
@@ -10412,7 +10412,7 @@
       </c>
       <c r="P132" s="4" t="inlineStr">
         <is>
-          <t>2210 (99.50%)</t>
+          <t>2215 (99.51%)</t>
         </is>
       </c>
     </row>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="I133" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J133" s="4" t="inlineStr">
         <is>
@@ -10476,7 +10476,7 @@
       </c>
       <c r="N133" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O133" s="4" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="P133" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -10526,7 +10526,7 @@
         </is>
       </c>
       <c r="I134" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J134" s="4" t="inlineStr">
         <is>
@@ -10560,7 +10560,7 @@
       </c>
       <c r="P134" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -10600,7 +10600,7 @@
         </is>
       </c>
       <c r="I135" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J135" s="4" t="inlineStr">
         <is>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="P135" s="4" t="inlineStr">
         <is>
-          <t>2213 (99.64%)</t>
+          <t>2218 (99.64%)</t>
         </is>
       </c>
     </row>
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="I136" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J136" s="4" t="inlineStr">
         <is>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="P136" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -10748,7 +10748,7 @@
         </is>
       </c>
       <c r="I137" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J137" s="4" t="inlineStr">
         <is>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="N137" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="O137" s="4" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="P137" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -10824,7 +10824,7 @@
         </is>
       </c>
       <c r="I138" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J138" s="4" t="inlineStr">
         <is>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="P138" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -10898,7 +10898,7 @@
         </is>
       </c>
       <c r="I139" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J139" s="4" t="inlineStr">
         <is>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="N139" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="O139" s="4" t="inlineStr">
@@ -10932,7 +10932,7 @@
       </c>
       <c r="P139" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -10972,7 +10972,7 @@
         </is>
       </c>
       <c r="I140" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J140" s="4" t="inlineStr">
         <is>
@@ -10986,7 +10986,7 @@
       </c>
       <c r="L140" s="4" t="inlineStr">
         <is>
-          <t>29 (1.31%)</t>
+          <t>29 (1.30%)</t>
         </is>
       </c>
       <c r="M140" s="4" t="inlineStr">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="N140" s="4" t="inlineStr">
         <is>
-          <t>94 (4.23%)</t>
+          <t>94 (4.22%)</t>
         </is>
       </c>
       <c r="O140" s="4" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="P140" s="4" t="inlineStr">
         <is>
-          <t>2094 (94.28%)</t>
+          <t>2099 (94.29%)</t>
         </is>
       </c>
     </row>
@@ -11042,7 +11042,7 @@
         </is>
       </c>
       <c r="I141" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J141" s="4" t="inlineStr">
         <is>
@@ -11056,7 +11056,7 @@
       </c>
       <c r="L141" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M141" s="4" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="N141" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O141" s="4" t="inlineStr">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="P141" s="4" t="inlineStr">
         <is>
-          <t>2219 (99.91%)</t>
+          <t>2224 (99.91%)</t>
         </is>
       </c>
     </row>
@@ -11112,7 +11112,7 @@
         </is>
       </c>
       <c r="I142" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J142" s="4" t="inlineStr">
         <is>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="N142" s="4" t="inlineStr">
         <is>
-          <t>144 (6.48%)</t>
+          <t>144 (6.47%)</t>
         </is>
       </c>
       <c r="O142" s="4" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="P142" s="4" t="inlineStr">
         <is>
-          <t>2077 (93.52%)</t>
+          <t>2082 (93.53%)</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="I143" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J143" s="4" t="inlineStr">
         <is>
@@ -11220,7 +11220,7 @@
       </c>
       <c r="P143" s="4" t="inlineStr">
         <is>
-          <t>2211 (99.55%)</t>
+          <t>2216 (99.55%)</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11256,7 @@
         </is>
       </c>
       <c r="I144" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J144" s="4" t="inlineStr">
         <is>
@@ -11270,7 +11270,7 @@
       </c>
       <c r="L144" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M144" s="4" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="N144" s="4" t="inlineStr">
         <is>
-          <t>11 (0.50%)</t>
+          <t>11 (0.49%)</t>
         </is>
       </c>
       <c r="O144" s="4" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="P144" s="4" t="inlineStr">
         <is>
-          <t>2209 (99.46%)</t>
+          <t>2214 (99.46%)</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="I145" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J145" s="4" t="inlineStr">
         <is>
@@ -11339,7 +11339,7 @@
       </c>
       <c r="K145" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L145" s="4" t="inlineStr">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="P145" s="4" t="inlineStr">
         <is>
-          <t>2200 (99.05%)</t>
+          <t>2205 (99.06%)</t>
         </is>
       </c>
     </row>
@@ -11404,7 +11404,7 @@
         </is>
       </c>
       <c r="I146" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J146" s="4" t="inlineStr">
         <is>
@@ -11438,7 +11438,7 @@
       </c>
       <c r="P146" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -11478,7 +11478,7 @@
         </is>
       </c>
       <c r="I147" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J147" s="4" t="inlineStr">
         <is>
@@ -11492,7 +11492,7 @@
       </c>
       <c r="L147" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="M147" s="4" t="inlineStr">
@@ -11512,7 +11512,7 @@
       </c>
       <c r="P147" s="4" t="inlineStr">
         <is>
-          <t>2216 (99.77%)</t>
+          <t>2221 (99.78%)</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
         </is>
       </c>
       <c r="I148" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J148" s="4" t="inlineStr">
         <is>
@@ -11576,7 +11576,7 @@
       </c>
       <c r="N148" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="O148" s="4" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="P148" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -11622,7 +11622,7 @@
         </is>
       </c>
       <c r="I149" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J149" s="4" t="inlineStr">
         <is>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="K149" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L149" s="4" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="P149" s="4" t="inlineStr">
         <is>
-          <t>2218 (99.86%)</t>
+          <t>2223 (99.87%)</t>
         </is>
       </c>
     </row>
@@ -11696,7 +11696,7 @@
         </is>
       </c>
       <c r="I150" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J150" s="4" t="inlineStr">
         <is>
@@ -11705,7 +11705,7 @@
       </c>
       <c r="K150" s="4" t="inlineStr">
         <is>
-          <t>3 (0.14%)</t>
+          <t>3 (0.13%)</t>
         </is>
       </c>
       <c r="L150" s="4" t="inlineStr">
@@ -11720,7 +11720,7 @@
       </c>
       <c r="N150" s="4" t="inlineStr">
         <is>
-          <t>72 (3.24%)</t>
+          <t>72 (3.23%)</t>
         </is>
       </c>
       <c r="O150" s="4" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="P150" s="4" t="inlineStr">
         <is>
-          <t>2128 (95.81%)</t>
+          <t>2133 (95.82%)</t>
         </is>
       </c>
     </row>
@@ -11770,7 +11770,7 @@
         </is>
       </c>
       <c r="I151" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J151" s="4" t="inlineStr">
         <is>
@@ -11804,7 +11804,7 @@
       </c>
       <c r="P151" s="4" t="inlineStr">
         <is>
-          <t>2197 (98.92%)</t>
+          <t>2202 (98.92%)</t>
         </is>
       </c>
     </row>
@@ -11844,7 +11844,7 @@
         </is>
       </c>
       <c r="I152" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J152" s="4" t="inlineStr">
         <is>
@@ -11878,7 +11878,7 @@
       </c>
       <c r="P152" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -11918,7 +11918,7 @@
         </is>
       </c>
       <c r="I153" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J153" s="4" t="inlineStr">
         <is>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="L153" s="4" t="inlineStr">
         <is>
-          <t>5 (0.23%)</t>
+          <t>5 (0.22%)</t>
         </is>
       </c>
       <c r="M153" s="4" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="P153" s="4" t="inlineStr">
         <is>
-          <t>2164 (97.43%)</t>
+          <t>2169 (97.44%)</t>
         </is>
       </c>
     </row>
@@ -11992,7 +11992,7 @@
         </is>
       </c>
       <c r="I154" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J154" s="4" t="inlineStr">
         <is>
@@ -12006,7 +12006,7 @@
       </c>
       <c r="L154" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="M154" s="4" t="inlineStr">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="N154" s="4" t="inlineStr">
         <is>
-          <t>80 (3.60%)</t>
+          <t>80 (3.59%)</t>
         </is>
       </c>
       <c r="O154" s="4" t="inlineStr">
@@ -12026,7 +12026,7 @@
       </c>
       <c r="P154" s="4" t="inlineStr">
         <is>
-          <t>2122 (95.54%)</t>
+          <t>2127 (95.55%)</t>
         </is>
       </c>
     </row>
@@ -12066,7 +12066,7 @@
         </is>
       </c>
       <c r="I155" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J155" s="4" t="inlineStr">
         <is>
@@ -12100,7 +12100,7 @@
       </c>
       <c r="P155" s="4" t="inlineStr">
         <is>
-          <t>2215 (99.73%)</t>
+          <t>2220 (99.73%)</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12140,7 @@
         </is>
       </c>
       <c r="I156" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J156" s="4" t="inlineStr">
         <is>
@@ -12164,7 +12164,7 @@
       </c>
       <c r="N156" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="O156" s="4" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="P156" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12214,7 @@
         </is>
       </c>
       <c r="I157" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J157" s="4" t="inlineStr">
         <is>
@@ -12248,7 +12248,7 @@
       </c>
       <c r="P157" s="4" t="inlineStr">
         <is>
-          <t>2209 (99.46%)</t>
+          <t>2214 (99.46%)</t>
         </is>
       </c>
     </row>
@@ -12288,7 +12288,7 @@
         </is>
       </c>
       <c r="I158" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J158" s="4" t="inlineStr">
         <is>
@@ -12297,7 +12297,7 @@
       </c>
       <c r="K158" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="L158" s="4" t="inlineStr">
@@ -12322,7 +12322,7 @@
       </c>
       <c r="P158" s="4" t="inlineStr">
         <is>
-          <t>2198 (98.96%)</t>
+          <t>2203 (98.97%)</t>
         </is>
       </c>
     </row>
@@ -12362,7 +12362,7 @@
         </is>
       </c>
       <c r="I159" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J159" s="4" t="inlineStr">
         <is>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="P159" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -12432,7 +12432,7 @@
         </is>
       </c>
       <c r="I160" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J160" s="4" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="M160" s="4" t="inlineStr">
         <is>
-          <t>1 (0.05%)</t>
+          <t>1 (0.04%)</t>
         </is>
       </c>
       <c r="N160" s="4" t="inlineStr">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="P160" s="4" t="inlineStr">
         <is>
-          <t>2220 (99.95%)</t>
+          <t>2225 (99.96%)</t>
         </is>
       </c>
     </row>
@@ -12506,7 +12506,7 @@
         </is>
       </c>
       <c r="I161" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J161" s="4" t="inlineStr">
         <is>
@@ -12540,7 +12540,7 @@
       </c>
       <c r="P161" s="4" t="inlineStr">
         <is>
-          <t>2215 (99.73%)</t>
+          <t>2220 (99.73%)</t>
         </is>
       </c>
     </row>
@@ -12576,7 +12576,7 @@
         </is>
       </c>
       <c r="I162" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J162" s="4" t="inlineStr">
         <is>
@@ -12600,7 +12600,7 @@
       </c>
       <c r="N162" s="4" t="inlineStr">
         <is>
-          <t>111 (5.00%)</t>
+          <t>111 (4.99%)</t>
         </is>
       </c>
       <c r="O162" s="4" t="inlineStr">
@@ -12610,7 +12610,7 @@
       </c>
       <c r="P162" s="4" t="inlineStr">
         <is>
-          <t>2106 (94.82%)</t>
+          <t>2111 (94.83%)</t>
         </is>
       </c>
     </row>
@@ -12650,7 +12650,7 @@
         </is>
       </c>
       <c r="I163" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J163" s="4" t="inlineStr">
         <is>
@@ -12674,7 +12674,7 @@
       </c>
       <c r="N163" s="4" t="inlineStr">
         <is>
-          <t>51 (2.30%)</t>
+          <t>51 (2.29%)</t>
         </is>
       </c>
       <c r="O163" s="4" t="inlineStr">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="P163" s="4" t="inlineStr">
         <is>
-          <t>2170 (97.70%)</t>
+          <t>2175 (97.71%)</t>
         </is>
       </c>
     </row>
@@ -12720,7 +12720,7 @@
         </is>
       </c>
       <c r="I164" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J164" s="4" t="inlineStr">
         <is>
@@ -12739,12 +12739,12 @@
       </c>
       <c r="M164" s="4" t="inlineStr">
         <is>
-          <t>13 (0.59%)</t>
+          <t>13 (0.58%)</t>
         </is>
       </c>
       <c r="N164" s="4" t="inlineStr">
         <is>
-          <t>151 (6.80%)</t>
+          <t>151 (6.78%)</t>
         </is>
       </c>
       <c r="O164" s="4" t="inlineStr">
@@ -12754,7 +12754,7 @@
       </c>
       <c r="P164" s="4" t="inlineStr">
         <is>
-          <t>2033 (91.54%)</t>
+          <t>2038 (91.55%)</t>
         </is>
       </c>
     </row>
@@ -12794,7 +12794,7 @@
         </is>
       </c>
       <c r="I165" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J165" s="4" t="inlineStr">
         <is>
@@ -12828,7 +12828,7 @@
       </c>
       <c r="P165" s="4" t="inlineStr">
         <is>
-          <t>2221 (100.00%)</t>
+          <t>2226 (100.00%)</t>
         </is>
       </c>
     </row>
@@ -12864,7 +12864,7 @@
         </is>
       </c>
       <c r="I166" s="4" t="n">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="J166" s="4" t="inlineStr">
         <is>
@@ -12888,7 +12888,7 @@
       </c>
       <c r="N166" s="4" t="inlineStr">
         <is>
-          <t>7 (0.32%)</t>
+          <t>7 (0.31%)</t>
         </is>
       </c>
       <c r="O166" s="4" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="P166" s="4" t="inlineStr">
         <is>
-          <t>2214 (99.68%)</t>
+          <t>2219 (99.69%)</t>
         </is>
       </c>
     </row>
@@ -13264,7 +13264,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -13276,25 +13276,25 @@
         <v>16</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>1.5209</v>
+        <v>1.5137</v>
       </c>
       <c r="H3" t="n">
         <v>57</v>
       </c>
       <c r="I3" s="8" t="n">
-        <v>5.4183</v>
+        <v>5.3926</v>
       </c>
       <c r="J3" t="n">
         <v>21</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>1.9962</v>
+        <v>1.9868</v>
       </c>
       <c r="L3" t="n">
         <v>299</v>
       </c>
       <c r="M3" s="8" t="n">
-        <v>28.4221</v>
+        <v>28.2876</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
@@ -13303,10 +13303,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="Q3" s="8" t="n">
-        <v>62.6426</v>
+        <v>62.8193</v>
       </c>
     </row>
     <row r="4">
@@ -13549,7 +13549,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -13567,19 +13567,19 @@
         <v>11</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>1.0456</v>
+        <v>1.0407</v>
       </c>
       <c r="J8" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>0.3802</v>
+        <v>0.3784</v>
       </c>
       <c r="L8" t="n">
         <v>116</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>11.0266</v>
+        <v>10.9745</v>
       </c>
       <c r="N8" t="n">
         <v>0</v>
@@ -13588,10 +13588,10 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>87.5475</v>
+        <v>87.60639999999999</v>
       </c>
     </row>
     <row r="9">
@@ -13834,7 +13834,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -13846,25 +13846,25 @@
         <v>16</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>1.5209</v>
+        <v>1.5137</v>
       </c>
       <c r="H13" t="n">
         <v>70</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>6.654</v>
+        <v>6.6225</v>
       </c>
       <c r="J13" t="n">
         <v>20</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>1.9011</v>
+        <v>1.8921</v>
       </c>
       <c r="L13" t="n">
         <v>272</v>
       </c>
       <c r="M13" s="8" t="n">
-        <v>25.8555</v>
+        <v>25.7332</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -13873,10 +13873,10 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="Q13" s="8" t="n">
-        <v>64.0684</v>
+        <v>64.2384</v>
       </c>
     </row>
     <row r="14">

</xml_diff>